<commit_message>
Memoria v3: agrega viento, columnas (esbeltez), refuerzo escalera; corrige vigas VC/VR con envolvente y longitudes de desarrollo
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/DISENO-ESCALERA.xlsx
+++ b/Proyectos/Diseno-Estructural/DISENO-ESCALERA.xlsx
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>0.125</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="9">
@@ -666,7 +666,7 @@
       </c>
       <c r="B20" s="6">
         <f>B7*B8/COS(RADIANS(B11))</f>
-        <v>4.242640687</v>
+        <v>4.412346315</v>
       </c>
     </row>
     <row r="21">
@@ -708,7 +708,7 @@
       </c>
       <c r="B24" s="8">
         <f>B20+B21+B22+B23</f>
-        <v>9.242640687</v>
+        <v>9.412346315</v>
       </c>
     </row>
     <row r="25">
@@ -729,7 +729,7 @@
       </c>
       <c r="B26" s="8">
         <f>1.2*B24+1.6*B25</f>
-        <v>15.89116882</v>
+        <v>16.09481558</v>
       </c>
     </row>
     <row r="28">
@@ -747,7 +747,7 @@
       </c>
       <c r="B29" s="6">
         <f>B7*B8</f>
-        <v>3</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="30">
@@ -778,7 +778,7 @@
       </c>
       <c r="B32" s="8">
         <f>B29+B30+B31</f>
-        <v>4.2</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="33">
@@ -789,7 +789,7 @@
       </c>
       <c r="B33" s="8">
         <f>1.2*B32+1.6*B25</f>
-        <v>9.84</v>
+        <v>9.984</v>
       </c>
     </row>
     <row r="35">
@@ -807,7 +807,7 @@
       </c>
       <c r="B36" s="9">
         <f>B26*B17^2/8</f>
-        <v>12.41497564</v>
+        <v>12.57407467</v>
       </c>
     </row>
     <row r="37">
@@ -818,7 +818,7 @@
       </c>
       <c r="B37" s="9">
         <f>B26*B17/2</f>
-        <v>19.86396103</v>
+        <v>20.11851947</v>
       </c>
     </row>
     <row r="39">
@@ -836,7 +836,7 @@
       </c>
       <c r="B40" s="10">
         <f>B8*1000-B12*1000-B13/2</f>
-        <v>93.65</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="41">
@@ -847,7 +847,7 @@
       </c>
       <c r="B41" s="6">
         <f>B36*1000000/(0.9*1000*B40^2)</f>
-        <v>1.572851783</v>
+        <v>1.435619492</v>
       </c>
     </row>
     <row r="42">
@@ -858,7 +858,7 @@
       </c>
       <c r="B42" s="11">
         <f>(0.85*B5/B6)*(1-SQRT(1-2*B41/(0.85*B5)))</f>
-        <v>0.003877550471</v>
+        <v>0.00352796397</v>
       </c>
     </row>
     <row r="43">
@@ -869,7 +869,7 @@
       </c>
       <c r="B43" s="12">
         <f>B42*1000*B40</f>
-        <v>363.1326016</v>
+        <v>348.0336457</v>
       </c>
     </row>
     <row r="44">
@@ -880,7 +880,7 @@
       </c>
       <c r="B44" s="12">
         <f>MAX(0.0018*1000*B8*1000,MAX(0.25*SQRT(B5)/B6,1.4/B6)*1000*B40)</f>
-        <v>312.1666667</v>
+        <v>328.8333333</v>
       </c>
     </row>
     <row r="45">
@@ -891,7 +891,7 @@
       </c>
       <c r="B45" s="13">
         <f>MAX(B43,B44)</f>
-        <v>363.1326016</v>
+        <v>348.0336457</v>
       </c>
     </row>
     <row r="46">
@@ -902,7 +902,7 @@
       </c>
       <c r="B46" s="12">
         <f>B14*1000/B45</f>
-        <v>355.2421331</v>
+        <v>370.6538193</v>
       </c>
     </row>
     <row r="47">
@@ -913,7 +913,7 @@
       </c>
       <c r="B47" s="12">
         <f>MIN(3*B8*1000,450)</f>
-        <v>375</v>
+        <v>390</v>
       </c>
     </row>
     <row r="48">
@@ -943,7 +943,7 @@
       </c>
       <c r="B51" s="12">
         <f>0.0018*1000*B8*1000</f>
-        <v>225</v>
+        <v>234</v>
       </c>
     </row>
     <row r="52">
@@ -984,7 +984,7 @@
       </c>
       <c r="B56" s="10">
         <f>0.75*0.17*SQRT(B5)*1000*B40/1000</f>
-        <v>63.18252562</v>
+        <v>66.55585854</v>
       </c>
     </row>
     <row r="57">

</xml_diff>